<commit_message>
Remove department field from database models, API, and UI
</commit_message>
<xml_diff>
--- a/sample_motors.xlsx
+++ b/sample_motors.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF18"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,145 +434,140 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Department</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Voltage</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Voltage</t>
+          <t>Current</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>RPM</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>RPM</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>Motor Make</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Motor Make</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Serial Number</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Serial Number</t>
+          <t>Frame</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Frame</t>
+          <t>Duty</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Duty</t>
+          <t>Protection</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Protection</t>
+          <t>Insulation</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Insulation</t>
+          <t>MCC</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>MCC</t>
+          <t>Feeder</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>Feeder</t>
+          <t>PCC</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>PCC</t>
+          <t>Substation</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Substation</t>
+          <t>Incoming</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Incoming</t>
+          <t>Cable Size</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Cable Size</t>
+          <t>Cable Length</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Cable Length</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Drawing Link</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>Drawing Link</t>
+          <t>Image Link</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Image Link</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Commission Date</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>Commission Date</t>
+          <t>Last Maintenance Date</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>Last Maintenance Date</t>
+          <t>Next Maintenance Date</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
-        <is>
-          <t>Next Maintenance Date</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
         <is>
           <t>Is Critical</t>
         </is>
@@ -596,143 +591,138 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>110 kW</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>110 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
           <t>190 A</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="G2" t="n">
         <v>1485</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>94.5%</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>94.5%</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>1LA8315-4AB60</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1LA8315-4AB60</t>
+          <t>S-98481A22</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>S-98481A22</t>
+          <t>315M</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>315M</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>MCC-1</t>
+          <t>Feeder-1</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Feeder-1</t>
+          <t>PCC-1</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>PCC-1</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 185 sq mm Al</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>3C x 185 sq mm Al</t>
+          <t>120 m</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>120 m</t>
+          <t>CHP Incline Gantry</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CHP Incline Gantry</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Primary coal transport drive. Critical equipment.</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Primary coal transport drive. Critical equipment.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2022-04-12</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>2022-04-12</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -756,143 +746,138 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>250 kW</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>250 kW</t>
+          <t>3300 V</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3300 V</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
           <t>55 A</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="G3" t="n">
         <v>990</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>95.2%</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>95.2%</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>M3BP-355MLA</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>M3BP-355MLA</t>
+          <t>A-83921B19</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>A-83921B19</t>
+          <t>355ML</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>355ML</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP56</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>IP56</t>
+          <t>Class H</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Class H</t>
+          <t>MCC-1</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>MCC-1</t>
+          <t>Feeder-2</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Feeder-2</t>
+          <t>PCC-1</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>PCC-1</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 95 sq mm Cu</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>3C x 95 sq mm Cu</t>
+          <t>80 m</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>80 m</t>
+          <t>Crusher House Level 2</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Crusher House Level 2</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>HT motor. High vibration area.</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>HT motor. High vibration area.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2022-05-01</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2022-05-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
-        <is>
-          <t>2026-12-15</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -916,143 +901,138 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>22 kW</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>22 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
           <t>39 A</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="G4" t="n">
         <v>1460</v>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>91.8%</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>91.8%</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>1LE1001-1DB4</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1LE1001-1DB4</t>
+          <t>S-38291C01</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>S-38291C01</t>
+          <t>160L</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>160L</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-1</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>MCC-1</t>
+          <t>Feeder-3</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Feeder-3</t>
+          <t>PCC-1</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>PCC-1</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 25 sq mm Al</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>3C x 25 sq mm Al</t>
+          <t>150 m</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>150 m</t>
+          <t>Crusher House Level 1</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>Crusher House Level 1</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Standard LT drive. Subject to high mechanical vibration.</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>Standard LT drive. Subject to high mechanical vibration.</t>
+          <t>Standby</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Standby</t>
+          <t>2022-04-15</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>2022-04-15</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1076,143 +1056,138 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>45 kW</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>45 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
           <t>78 A</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="G5" t="n">
         <v>1475</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>93.6%</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>93.6%</t>
+          <t>CG Global</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>CG Global</t>
+          <t>GD180L</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>GD180L</t>
+          <t>C-1293810</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>C-1293810</t>
+          <t>225M</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>225M</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-1</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>MCC-1</t>
+          <t>Feeder-4</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Feeder-4</t>
+          <t>PCC-1</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>PCC-1</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 50 sq mm Al</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>3C x 50 sq mm Al</t>
+          <t>110 m</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>110 m</t>
+          <t>Bag Filter Area</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Bag Filter Area</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>VFD driven for speed control. Interlocked with Crusher.</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>VFD driven for speed control. Interlocked with Crusher.</t>
+          <t>Fault</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Fault</t>
+          <t>2022-04-18</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>2022-04-18</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1236,143 +1211,138 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>630 kW</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>630 kW</t>
+          <t>6600 V</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>6600 V</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
           <t>68 A</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="G6" t="n">
         <v>2980</v>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>96.1%</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>96.1%</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>AMI-500L2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AMI-500L2</t>
+          <t>A-72819C20</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>A-72819C20</t>
+          <t>500L</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>500L</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class H</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Class H</t>
+          <t>MCC-2</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>MCC-2</t>
+          <t>Feeder-1</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Feeder-1</t>
+          <t>PCC-1</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>PCC-1</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 120 sq mm Cu</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>3C x 120 sq mm Cu</t>
+          <t>210 m</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>210 m</t>
+          <t>Boiler House Pump Floor</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Boiler House Pump Floor</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Ultra-critical HT pump. Subject to strict thermal monitoring.</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Ultra-critical HT pump. Subject to strict thermal monitoring.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2021-10-10</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>2021-10-10</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="AF6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1396,143 +1366,138 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>630 kW</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>630 kW</t>
+          <t>6600 V</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>6600 V</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
           <t>68 A</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="G7" t="n">
         <v>2980</v>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>96.1%</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>96.1%</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>AMI-500L2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>AMI-500L2</t>
+          <t>A-72819C21</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>A-72819C21</t>
+          <t>500L</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>500L</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class H</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Class H</t>
+          <t>MCC-2</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>MCC-2</t>
+          <t>Feeder-2</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Feeder-2</t>
+          <t>PCC-1</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>PCC-1</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 120 sq mm Cu</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>3C x 120 sq mm Cu</t>
+          <t>215 m</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>215 m</t>
+          <t>Boiler House Pump Floor</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Boiler House Pump Floor</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Standby feed pump. Ready for auto-changeover.</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>Standby feed pump. Ready for auto-changeover.</t>
+          <t>Standby</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>Standby</t>
+          <t>2021-10-12</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>2021-10-12</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="AF7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1556,143 +1521,138 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>132 kW</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>132 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
           <t>225 A</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="G8" t="n">
         <v>1485</v>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>94.8%</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>94.8%</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>1LA8315-4AB60</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1LA8315-4AB60</t>
+          <t>S-22819C</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>S-22819C</t>
+          <t>315M</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>315M</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-2</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>MCC-2</t>
+          <t>Feeder-3</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Feeder-3</t>
+          <t>PCC-1</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>PCC-1</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 240 sq mm Al</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>3C x 240 sq mm Al</t>
+          <t>90 m</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>90 m</t>
+          <t>Boiler Draft Fan Floor</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Boiler Draft Fan Floor</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Forced Draft fan. VFD speed controller active.</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Forced Draft fan. VFD speed controller active.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2021-11-20</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2021-11-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-12-22</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
-        <is>
-          <t>2026-12-22</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1716,143 +1676,138 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>90 kW</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>90 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
           <t>155 A</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="G9" t="n">
         <v>1475</v>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>93.9%</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>93.9%</t>
+          <t>CG Global</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>CG Global</t>
+          <t>GD250M</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>GD250M</t>
+          <t>C-39102</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>C-39102</t>
+          <t>280S</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>280S</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-3</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>MCC-3</t>
+          <t>Feeder-1</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Feeder-1</t>
+          <t>PCC-2</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>PCC-2</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 185 sq mm Al</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>3C x 185 sq mm Al</t>
+          <t>65 m</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>65 m</t>
+          <t>Cooling Tower Basin Area</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Cooling Tower Basin Area</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Continuous circulation duty.</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Continuous circulation duty.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2022-01-15</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>2022-01-15</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-      <c r="AF9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1876,143 +1831,138 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>90 kW</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>90 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
           <t>155 A</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="G10" t="n">
         <v>1475</v>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>93.9%</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>93.9%</t>
+          <t>CG Global</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>CG Global</t>
+          <t>GD250M</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>GD250M</t>
+          <t>C-39103</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>C-39103</t>
+          <t>280S</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>280S</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-3</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>MCC-3</t>
+          <t>Feeder-2</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Feeder-2</t>
+          <t>PCC-2</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>PCC-2</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 185 sq mm Al</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>3C x 185 sq mm Al</t>
+          <t>70 m</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>70 m</t>
+          <t>Cooling Tower Basin Area</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Cooling Tower Basin Area</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Standby circulation pump.</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Standby circulation pump.</t>
+          <t>Standby</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Standby</t>
+          <t>2022-01-18</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>2022-01-18</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
-        <is>
-          <t>2026-11-15</t>
-        </is>
-      </c>
-      <c r="AF10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2036,143 +1986,138 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>30 kW</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>30 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
           <t>53 A</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="G11" t="n">
         <v>970</v>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>92.4%</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>92.4%</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>1LE1001-2DB4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1LE1001-2DB4</t>
+          <t>S-38291</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>S-38291</t>
+          <t>200L</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>200L</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP56</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>IP56</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-3</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>MCC-3</t>
+          <t>Feeder-3</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Feeder-3</t>
+          <t>PCC-2</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>PCC-2</t>
+          <t>Main Substation-1</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Main Substation-1</t>
+          <t>33kV Incoming-1</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>33kV Incoming-1</t>
+          <t>3C x 35 sq mm Al</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>3C x 35 sq mm Al</t>
+          <t>85 m</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>85 m</t>
+          <t>Cooling Tower Fan Deck</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Cooling Tower Fan Deck</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Exhaust fan. Humidity exposed bearings.</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Exhaust fan. Humidity exposed bearings.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2022-01-20</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>2022-01-20</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-12-10</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="AF11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2196,143 +2141,138 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>160 kW</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>160 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
           <t>270 A</t>
         </is>
       </c>
-      <c r="H12" t="n">
+      <c r="G12" t="n">
         <v>1485</v>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>95.0%</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>M3BP-315MLA</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>M3BP-315MLA</t>
+          <t>A-9281A</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>A-9281A</t>
+          <t>315S</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>315S</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-4</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>MCC-4</t>
+          <t>Feeder-1</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Feeder-1</t>
+          <t>PCC-4</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>PCC-4</t>
+          <t>Main Substation-2</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Main Substation-2</t>
+          <t>33kV Incoming-2</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>33kV Incoming-2</t>
+          <t>3C x 300 sq mm Al</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>3C x 300 sq mm Al</t>
+          <t>60 m</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>60 m</t>
+          <t>Utility Compressor Room</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Utility Compressor Room</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Star-Delta starter. Clean dry environment.</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Star-Delta starter. Clean dry environment.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2023-02-15</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>2023-02-15</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="AF12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2356,143 +2296,138 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>160 kW</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>160 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
           <t>270 A</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="G13" t="n">
         <v>1485</v>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>95.0%</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>95.0%</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>M3BP-315MLA</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>M3BP-315MLA</t>
+          <t>A-9281B</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>A-9281B</t>
+          <t>315S</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>315S</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-4</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>MCC-4</t>
+          <t>Feeder-2</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Feeder-2</t>
+          <t>PCC-4</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>PCC-4</t>
+          <t>Main Substation-2</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Main Substation-2</t>
+          <t>33kV Incoming-2</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>33kV Incoming-2</t>
+          <t>3C x 300 sq mm Al</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>3C x 300 sq mm Al</t>
+          <t>65 m</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>65 m</t>
+          <t>Utility Compressor Room</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Utility Compressor Room</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Standby compressor.</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Standby compressor.</t>
+          <t>Standby</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>Standby</t>
+          <t>2023-02-18</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>2023-02-18</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="AF13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2516,143 +2451,138 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>200 kW</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>200 kW</t>
+          <t>3300 V</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3300 V</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
           <t>44 A</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="G14" t="n">
         <v>1480</v>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>94.8%</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>94.8%</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>1LA8315-4AB60</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1LA8315-4AB60</t>
+          <t>S-38102A</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>S-38102A</t>
+          <t>315L</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>315L</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-5</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>MCC-5</t>
+          <t>Feeder-1</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Feeder-1</t>
+          <t>PCC-5</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>PCC-5</t>
+          <t>Main Substation-2</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Main Substation-2</t>
+          <t>33kV Incoming-2</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>33kV Incoming-2</t>
+          <t>3C x 95 sq mm Al</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>3C x 95 sq mm Al</t>
+          <t>350 m</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>350 m</t>
+          <t>River Intake Pump House</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>River Intake Pump House</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>High static head, remote location.</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>High static head, remote location.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2023-05-10</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>2023-05-10</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
-        <is>
-          <t>2026-11-02</t>
-        </is>
-      </c>
-      <c r="AF14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -2676,143 +2606,138 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>11 kW</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
           <t>21 A</t>
         </is>
       </c>
-      <c r="H15" t="n">
+      <c r="G15" t="n">
         <v>960</v>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>89.5%</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>89.5%</t>
+          <t>CG Global</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>CG Global</t>
+          <t>GD160M</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>GD160M</t>
+          <t>C-29381A</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>C-29381A</t>
+          <t>160M</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>160M</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-5</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>MCC-5</t>
+          <t>Feeder-2</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Feeder-2</t>
+          <t>PCC-5</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>PCC-5</t>
+          <t>Main Substation-2</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Main Substation-2</t>
+          <t>33kV Incoming-2</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>33kV Incoming-2</t>
+          <t>3C x 10 sq mm Al</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>3C x 10 sq mm Al</t>
+          <t>80 m</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>80 m</t>
+          <t>Clarifier Tank 1</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Clarifier Tank 1</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Geared motor. High torque application.</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Geared motor. High torque application.</t>
+          <t>Fault</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>Fault</t>
+          <t>2023-05-15</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>2023-05-15</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="AF15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2836,143 +2761,138 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>37 kW</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>37 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
           <t>66 A</t>
         </is>
       </c>
-      <c r="H16" t="n">
+      <c r="G16" t="n">
         <v>2930</v>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>93.0%</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>93.0%</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>1LE1001-2AB4</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1LE1001-2AB4</t>
+          <t>S-38102B</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>S-38102B</t>
+          <t>200L</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>200L</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-5</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>MCC-5</t>
+          <t>Feeder-3</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Feeder-3</t>
+          <t>PCC-5</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>PCC-5</t>
+          <t>Main Substation-2</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Main Substation-2</t>
+          <t>33kV Incoming-2</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>33kV Incoming-2</t>
+          <t>3C x 35 sq mm Al</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>3C x 35 sq mm Al</t>
+          <t>120 m</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>120 m</t>
+          <t>Filter House Basement</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Filter House Basement</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Used during backwash cycle only. Soft Starter equipped.</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>Used during backwash cycle only. Soft Starter equipped.</t>
+          <t>Standby</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>Standby</t>
+          <t>2023-05-20</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>2023-05-20</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="AF16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2996,143 +2916,138 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>15 kW</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>15 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
           <t>28 A</t>
         </is>
       </c>
-      <c r="H17" t="n">
+      <c r="G17" t="n">
         <v>1440</v>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>90.2%</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>90.2%</t>
+          <t>CG Global</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>CG Global</t>
+          <t>GD160M</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>GD160M</t>
+          <t>C-29381B</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>C-29381B</t>
+          <t>160M</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>160M</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP55</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>IP55</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-6</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>MCC-6</t>
+          <t>Feeder-1</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Feeder-1</t>
+          <t>PCC-6</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>PCC-6</t>
+          <t>Utility Substation</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Utility Substation</t>
+          <t>33kV Utility Incomer</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>33kV Utility Incomer</t>
+          <t>3C x 16 sq mm Al</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>3C x 16 sq mm Al</t>
+          <t>45 m</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>45 m</t>
+          <t>ETP Pump Area</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>ETP Pump Area</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>ETP plant water transfer pump.</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>ETP plant water transfer pump.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2024-01-10</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>2024-01-10</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="AE17" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="AF17" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3156,143 +3071,138 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mechanical</t>
+          <t>22 kW</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>22 kW</t>
+          <t>415 V</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>415 V</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
           <t>39 A</t>
         </is>
       </c>
-      <c r="H18" t="n">
+      <c r="G18" t="n">
         <v>1450</v>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>91.5%</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>91.5%</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>1LE1001-1DB4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1LE1001-1DB4</t>
+          <t>S-9281C</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>S-9281C</t>
+          <t>180M</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>180M</t>
+          <t>S1 Continuous</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>S1 Continuous</t>
+          <t>IP56</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>IP56</t>
+          <t>Class F</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Class F</t>
+          <t>MCC-6</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>MCC-6</t>
+          <t>Feeder-2</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Feeder-2</t>
+          <t>PCC-6</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>PCC-6</t>
+          <t>Utility Substation</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Utility Substation</t>
+          <t>33kV Utility Incomer</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>33kV Utility Incomer</t>
+          <t>3C x 25 sq mm Al</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>3C x 25 sq mm Al</t>
+          <t>50 m</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>50 m</t>
+          <t>ETP Aeration Lagoon</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>ETP Aeration Lagoon</t>
+          <t>ga_motor.svg</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>ga_motor.svg</t>
+          <t>motor_photograph.svg</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>motor_photograph.svg</t>
+          <t>Outdoor installation. High humidity exposure.</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Outdoor installation. High humidity exposure.</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>2024-01-12</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>2024-01-12</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-11-18</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="AF18" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>